<commit_message>
UI fixes, Auth Context updates, and Shop Payment strict 2-step verification flow
</commit_message>
<xml_diff>
--- a/sample_20_students_fee.xlsx
+++ b/sample_20_students_fee.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9857F440-CD22-463C-9215-C830206F24DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B534D1D1-03CD-4252-983D-5F15EDDCF00C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -78,7 +78,7 @@
     <t>Summer</t>
   </si>
   <si>
-    <t>Summer 2026 Semester Fee</t>
+    <t>Summer 2028 Semester Fee</t>
   </si>
 </sst>
 </file>
@@ -533,13 +533,13 @@
         <v>15</v>
       </c>
       <c r="G2">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="H2">
         <v>45500</v>
       </c>
       <c r="I2" s="2">
-        <v>46233</v>
+        <v>46964</v>
       </c>
       <c r="J2" t="s">
         <v>16</v>

</xml_diff>